<commit_message>
2025 Feb 2025 resolved
</commit_message>
<xml_diff>
--- a/data/2025-02-Control_asistencia.xlsx
+++ b/data/2025-02-Control_asistencia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\OneDrive\Desktop\AsistenciaAsambleaLegislativa2022-2026\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2331E09C-8412-4DBC-A40C-57CEB986C45A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7959E22-C9FB-49EF-9D94-2D1825358339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="245" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -696,9 +696,7 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -830,38 +828,38 @@
     <xf numFmtId="1" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="24">
@@ -1226,94 +1224,94 @@
   <sheetData>
     <row r="1" spans="2:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:40" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="35" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="36" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="37" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="38" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" s="39" t="s">
+      <c r="B2" s="45" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="35" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="36" t="s">
         <v>68</v>
       </c>
-      <c r="G2" s="40" t="s">
+      <c r="G2" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="H2" s="41" t="s">
+      <c r="H2" s="38" t="s">
         <v>70</v>
       </c>
-      <c r="I2" s="41" t="s">
+      <c r="I2" s="43" t="s">
         <v>71</v>
       </c>
-      <c r="J2" s="42" t="s">
+      <c r="J2" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="K2" s="43" t="s">
+      <c r="K2" s="40" t="s">
         <v>73</v>
       </c>
-      <c r="L2" s="41" t="s">
+      <c r="L2" s="38" t="s">
         <v>74</v>
       </c>
-      <c r="M2" s="41" t="s">
+      <c r="M2" s="43" t="s">
         <v>75</v>
       </c>
-      <c r="N2" s="42" t="s">
+      <c r="N2" s="39" t="s">
         <v>76</v>
       </c>
-      <c r="O2" s="40" t="s">
+      <c r="O2" s="37" t="s">
         <v>77</v>
       </c>
-      <c r="P2" s="41" t="s">
+      <c r="P2" s="38" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="41" t="s">
+      <c r="Q2" s="43" t="s">
         <v>79</v>
       </c>
-      <c r="R2" s="44" t="s">
+      <c r="R2" s="41" t="s">
         <v>80</v>
       </c>
-      <c r="S2" s="40" t="s">
+      <c r="S2" s="37" t="s">
         <v>81</v>
       </c>
-      <c r="T2" s="45" t="s">
+      <c r="T2" s="44" t="s">
         <v>82</v>
       </c>
-      <c r="U2" s="42" t="s">
+      <c r="U2" s="39" t="s">
         <v>83</v>
       </c>
-      <c r="V2" s="43" t="s">
+      <c r="V2" s="40" t="s">
         <v>84</v>
       </c>
-      <c r="W2" s="41" t="s">
+      <c r="W2" s="43" t="s">
         <v>85</v>
       </c>
-      <c r="X2" s="42" t="s">
+      <c r="X2" s="39" t="s">
         <v>86</v>
       </c>
-      <c r="Y2" s="43" t="s">
+      <c r="Y2" s="40" t="s">
         <v>87</v>
       </c>
-      <c r="Z2" s="41" t="s">
+      <c r="Z2" s="38" t="s">
         <v>88</v>
       </c>
-      <c r="AA2" s="41" t="s">
+      <c r="AA2" s="43" t="s">
         <v>89</v>
       </c>
-      <c r="AB2" s="44" t="s">
+      <c r="AB2" s="41" t="s">
         <v>90</v>
       </c>
-      <c r="AC2" s="40" t="s">
+      <c r="AC2" s="37" t="s">
         <v>91</v>
       </c>
-      <c r="AD2" s="41" t="s">
+      <c r="AD2" s="43" t="s">
         <v>92</v>
       </c>
-      <c r="AE2" s="42" t="s">
+      <c r="AE2" s="39" t="s">
         <v>93</v>
       </c>
     </row>
@@ -6666,6 +6664,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101003025C3D639156D41ABE9029D7D6E875B" ma:contentTypeVersion="1" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a077238af601a547b4816ba50e6a1a48">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b14bbdcc-8c3b-45aa-839f-2124b15f3d4c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7dfb068e2175d5eef77397b40180d253" ns2:_="">
     <xsd:import namespace="b14bbdcc-8c3b-45aa-839f-2124b15f3d4c"/>
@@ -6805,15 +6812,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -6821,6 +6819,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{09776615-25AF-497F-B95C-60AE33983371}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AFD152A1-7FC2-4A9B-AA3C-B0EACDBD29EA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6838,14 +6844,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{09776615-25AF-497F-B95C-60AE33983371}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B0EB679-A57B-42F2-8493-FC2C0E0DADB0}">
   <ds:schemaRefs>

</xml_diff>